<commit_message>
Improve Part 2 classifier and upgrade report to full academic standard
- enrich ISIC division reference docs with full group/class vocabulary
  (isic_rev5_full.csv), improving match quality (e.g. N72 recall up)
- report: abstract, references, rigorous method, QDA spotlight,
  validation section with reproducible sample, data-quality and future work
- README: reflect 10 ECTS project scope, updated results and validation
</commit_message>
<xml_diff>
--- a/export/23293505-sq26-classification.xlsx
+++ b/export/23293505-sq26-classification.xlsx
@@ -508,7 +508,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>P84 Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -587,12 +587,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>P84 Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>R86 Human health activities</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>R87 Residential care activities</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -644,7 +644,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>P84 Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -672,7 +672,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>C18 Printing and reproduction of recorded media</t>
+          <t>T94 Activities of membership organizations</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -726,7 +726,11 @@
           <t>N73 Activities of advertising, market research and public relations</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>N72 Scientific research and development</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="n">
         <v>318</v>
       </c>
@@ -752,7 +756,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>L64 Financial service activities, except insurance and pension funding</t>
+          <t>L66 Activities auxiliary to financial service and insurance activities</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -775,14 +779,10 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>O82 Office administrative, office support and other business support activities</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>T94 Activities of membership organizations</t>
         </is>
       </c>
+      <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n">
         <v>23</v>
       </c>
@@ -808,7 +808,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>C15 Manufacture of leather and related products</t>
+          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
@@ -831,10 +831,14 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>R86 Human health activities</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
           <t>N71 Architectural and engineering activities; technical testing and analysis</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n">
         <v>3</v>
       </c>
@@ -886,11 +890,7 @@
           <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>K61 Telecommunications</t>
-        </is>
-      </c>
+      <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n">
         <v>21</v>
       </c>
@@ -911,12 +911,12 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>Q85 Education</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
           <t>O79 Travel agency, tour operator, and other travel related activities</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>U97 Activities of households as employers of domestic personnel</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
@@ -939,12 +939,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>N72 Scientific research and development</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
           <t>R86 Human health activities</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>R88 Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
@@ -991,12 +991,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>R88 Social work activities without accommodation</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>P84 Public administration and defence; compulsory social security</t>
+          <t>Q85 Education</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
@@ -1039,12 +1039,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
+          <t>O78 Employment activities</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
           <t>E39 Remediation and other waste management service activities</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>E37 Sewerage</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
@@ -1091,10 +1091,14 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
+          <t>O78 Employment activities</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
           <t>F42 Civil engineering</t>
         </is>
       </c>
-      <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n">
         <v>9</v>
       </c>
@@ -1139,10 +1143,14 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
+          <t>R86 Human health activities</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
           <t>R87 Residential care activities</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n">
         <v>6</v>
       </c>
@@ -1166,11 +1174,7 @@
           <t>J58 Publishing activities</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>J59 Motion picture, video and television programme production, sound recording and music publishing activities</t>
-        </is>
-      </c>
+      <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n">
         <v>55</v>
       </c>
@@ -1194,7 +1198,11 @@
           <t>N73 Activities of advertising, market research and public relations</t>
         </is>
       </c>
-      <c r="E28" s="2" t="n"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>N72 Scientific research and development</t>
+        </is>
+      </c>
       <c r="F28" s="2" t="n">
         <v>11</v>
       </c>
@@ -1218,11 +1226,7 @@
           <t>Q85 Education</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>T96 Personal service activities</t>
-        </is>
-      </c>
+      <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n">
         <v>62</v>
       </c>
@@ -1243,12 +1247,12 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
+          <t>N73 Activities of advertising, market research and public relations</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>D35 Electricity, gas, steam and air conditioning supply</t>
+          <t>P84 Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
@@ -1276,7 +1280,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>I56 Food and beverage service activities</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -1327,12 +1331,12 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>G46 Wholesale trade</t>
+          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>G47 Retail trade</t>
+          <t>O82 Office administrative, office support and other business support activities</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
@@ -1360,7 +1364,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>N72 Scientific research and development</t>
+          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -1416,7 +1420,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>C17 Manufacture of paper and paper products</t>
+          <t>O80 Investigation and security activities</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
@@ -1444,7 +1448,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>C17 Manufacture of paper and paper products</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -1470,7 +1474,11 @@
           <t>N73 Activities of advertising, market research and public relations</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>N72 Scientific research and development</t>
+        </is>
+      </c>
       <c r="F38" s="2" t="n">
         <v>161</v>
       </c>
@@ -1491,12 +1499,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
+          <t>T94 Activities of membership organizations</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
           <t>O78 Employment activities</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>G46 Wholesale trade</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
@@ -1572,7 +1580,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>T96 Personal service activities</t>
+          <t>I56 Food and beverage service activities</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
@@ -1626,11 +1634,7 @@
           <t>N72 Scientific research and development</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>O78 Employment activities</t>
-        </is>
-      </c>
+      <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n">
         <v>24</v>
       </c>
@@ -1651,12 +1655,12 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
+          <t>D35 Electricity, gas, steam and air conditioning supply</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
           <t>R86 Human health activities</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>R87 Residential care activities</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
@@ -1703,12 +1707,12 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
+          <t>Q85 Education</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
           <t>D35 Electricity, gas, steam and air conditioning supply</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>N71 Architectural and engineering activities; technical testing and analysis</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
@@ -1731,10 +1735,14 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>F43 Specialized construction activities</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="n"/>
+          <t>R86 Human health activities</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>R87 Residential care activities</t>
+        </is>
+      </c>
       <c r="F48" s="2" t="n">
         <v>28</v>
       </c>
@@ -1786,7 +1794,11 @@
           <t>F42 Civil engineering</t>
         </is>
       </c>
-      <c r="E50" s="2" t="n"/>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>N69 Legal and accounting activities</t>
+        </is>
+      </c>
       <c r="F50" s="2" t="n">
         <v>8</v>
       </c>
@@ -1836,7 +1848,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>R87 Residential care activities</t>
+          <t>U97 Activities of households as employers of domestic personnel</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
@@ -1879,14 +1891,10 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>T96 Personal service activities</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
           <t>Q85 Education</t>
         </is>
       </c>
+      <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="n">
         <v>64</v>
       </c>
@@ -1935,12 +1943,12 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
+          <t>S90 Arts creation and performing arts activities</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
           <t>C17 Manufacture of paper and paper products</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>S90 Arts creation and performing arts activities</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
@@ -1966,7 +1974,11 @@
           <t>C16 Manufacture of wood and of products of wood and cork, except furniture; manufacture of articles of straw and plaiting materials</t>
         </is>
       </c>
-      <c r="E57" s="2" t="n"/>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>E38 Waste collection, treatment and disposal, and recovery activities</t>
+        </is>
+      </c>
       <c r="F57" s="2" t="n">
         <v>90</v>
       </c>
@@ -2011,12 +2023,12 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>C18 Printing and reproduction of recorded media</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>R88 Social work activities without accommodation</t>
+          <t>R87 Residential care activities</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
@@ -2067,12 +2079,12 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>P84 Public administration and defence; compulsory social security</t>
+          <t>A03 Fishing and aquaculture</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>N73 Activities of advertising, market research and public relations</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
@@ -2147,14 +2159,10 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>N73 Activities of advertising, market research and public relations</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>N74 Other professional, scientific and technical activities</t>
-        </is>
-      </c>
+          <t>C30 Manufacture of other transport equipment</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n">
         <v>151</v>
       </c>
@@ -2206,7 +2214,11 @@
           <t>C21 Manufacture of basic pharmaceutical products and pharmaceutical preparations</t>
         </is>
       </c>
-      <c r="E66" s="2" t="n"/>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>L66 Activities auxiliary to financial service and insurance activities</t>
+        </is>
+      </c>
       <c r="F66" s="2" t="n">
         <v>5</v>
       </c>
@@ -2251,14 +2263,10 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>G46 Wholesale trade</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>G47 Retail trade</t>
-        </is>
-      </c>
+          <t>N72 Scientific research and development</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n">
         <v>941</v>
       </c>
@@ -2279,14 +2287,10 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>O82 Office administrative, office support and other business support activities</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>P84 Public administration and defence; compulsory social security</t>
-        </is>
-      </c>
+          <t>N73 Activities of advertising, market research and public relations</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="n"/>
       <c r="F69" s="2" t="n">
         <v>52</v>
       </c>
@@ -2307,12 +2311,12 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>C16 Manufacture of wood and of products of wood and cork, except furniture; manufacture of articles of straw and plaiting materials</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>C15 Manufacture of leather and related products</t>
+          <t>N71 Architectural and engineering activities; technical testing and analysis</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
@@ -2338,11 +2342,7 @@
           <t>Q85 Education</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>T96 Personal service activities</t>
-        </is>
-      </c>
+      <c r="E71" s="2" t="n"/>
       <c r="F71" s="2" t="n">
         <v>99</v>
       </c>
@@ -2363,7 +2363,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>R87 Residential care activities</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>Q85 Education</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Q85 Education</t>
+          <t>A03 Fishing and aquaculture</t>
         </is>
       </c>
       <c r="E74" s="2" t="n"/>
@@ -2467,12 +2467,12 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
+          <t>T94 Activities of membership organizations</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
           <t>J60 Programming, broadcasting, news agency and other content distribution activities</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>R88 Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
@@ -2522,11 +2522,7 @@
           <t>Q85 Education</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>T96 Personal service activities</t>
-        </is>
-      </c>
+      <c r="E78" s="2" t="n"/>
       <c r="F78" s="2" t="n">
         <v>63</v>
       </c>
@@ -2550,7 +2546,11 @@
           <t>J59 Motion picture, video and television programme production, sound recording and music publishing activities</t>
         </is>
       </c>
-      <c r="E79" s="2" t="n"/>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>B06 Extraction of crude petroleum and natural gas</t>
+        </is>
+      </c>
       <c r="F79" s="2" t="n">
         <v>32</v>
       </c>
@@ -2571,12 +2571,12 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>T96 Personal service activities</t>
+          <t>N73 Activities of advertising, market research and public relations</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
@@ -2627,12 +2627,12 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
+          <t>N72 Scientific research and development</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
           <t>J60 Programming, broadcasting, news agency and other content distribution activities</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>H50 Water transport</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>C16 Manufacture of wood and of products of wood and cork, except furniture; manufacture of articles of straw and plaiting materials</t>
+          <t>C32 Other manufacturing</t>
         </is>
       </c>
       <c r="E83" s="2" t="n"/>
@@ -2682,11 +2682,7 @@
           <t>Q85 Education</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>T96 Personal service activities</t>
-        </is>
-      </c>
+      <c r="E84" s="2" t="n"/>
       <c r="F84" s="2" t="n">
         <v>62</v>
       </c>
@@ -2710,11 +2706,7 @@
           <t>Q85 Education</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>T96 Personal service activities</t>
-        </is>
-      </c>
+      <c r="E85" s="2" t="n"/>
       <c r="F85" s="2" t="n">
         <v>61</v>
       </c>
@@ -2763,14 +2755,10 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>F43 Specialized construction activities</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>F41 Construction of residential and non-residential buildings</t>
-        </is>
-      </c>
+          <t>F42 Civil engineering</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n"/>
       <c r="F87" s="2" t="n">
         <v>52</v>
       </c>
@@ -2791,12 +2779,12 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>R88 Social work activities without accommodation</t>
+          <t>R87 Residential care activities</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>P84 Public administration and defence; compulsory social security</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
@@ -2852,7 +2840,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>V99 Activities of extraterritorial organizations and bodies</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
@@ -2934,11 +2922,7 @@
           <t>R86 Human health activities</t>
         </is>
       </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>R87 Residential care activities</t>
-        </is>
-      </c>
+      <c r="E93" s="2" t="n"/>
       <c r="F93" s="2" t="n">
         <v>3</v>
       </c>
@@ -2962,7 +2946,11 @@
           <t>N73 Activities of advertising, market research and public relations</t>
         </is>
       </c>
-      <c r="E94" s="2" t="n"/>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>N72 Scientific research and development</t>
+        </is>
+      </c>
       <c r="F94" s="2" t="n">
         <v>1533</v>
       </c>
@@ -2983,12 +2971,12 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>N73 Activities of advertising, market research and public relations</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>R88 Social work activities without accommodation</t>
+          <t>J60 Programming, broadcasting, news agency and other content distribution activities</t>
         </is>
       </c>
       <c r="F95" s="2" t="n">
@@ -3011,14 +2999,10 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>M68 Real estate activities</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>C15 Manufacture of leather and related products</t>
-        </is>
-      </c>
+          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="n"/>
       <c r="F96" s="2" t="n">
         <v>211</v>
       </c>
@@ -3039,7 +3023,7 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>O80 Investigation and security activities</t>
+          <t>P84 Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -3119,12 +3103,12 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>J58 Publishing activities</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>J60 Programming, broadcasting, news agency and other content distribution activities</t>
+          <t>A01 Crop and animal production, hunting and related service activities</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
@@ -3147,12 +3131,12 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
+          <t>K61 Telecommunications</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
           <t>R86 Human health activities</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>R87 Residential care activities</t>
         </is>
       </c>
       <c r="F101" s="2" t="n">
@@ -3247,12 +3231,12 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>A01 Crop and animal production, hunting and related service activities</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="F105" s="2" t="n">
@@ -3275,12 +3259,12 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>N69 Legal and accounting activities</t>
+          <t>N71 Architectural and engineering activities; technical testing and analysis</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>N71 Architectural and engineering activities; technical testing and analysis</t>
+          <t>C16 Manufacture of wood and of products of wood and cork, except furniture; manufacture of articles of straw and plaiting materials</t>
         </is>
       </c>
       <c r="F106" s="2" t="n">
@@ -3383,14 +3367,10 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>R88 Social work activities without accommodation</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
-        </is>
-      </c>
+          <t>D35 Electricity, gas, steam and air conditioning supply</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="n"/>
       <c r="F110" s="2" t="n">
         <v>116</v>
       </c>
@@ -3440,7 +3420,7 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="F112" s="2" t="n">
@@ -3463,7 +3443,7 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
@@ -3491,12 +3471,12 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>O82 Office administrative, office support and other business support activities</t>
+          <t>T96 Personal service activities</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>N74 Other professional, scientific and technical activities</t>
+          <t>E36 Water collection, treatment and supply</t>
         </is>
       </c>
       <c r="F114" s="2" t="n">
@@ -3544,7 +3524,7 @@
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>N72 Scientific research and development</t>
+          <t>N74 Other professional, scientific and technical activities</t>
         </is>
       </c>
       <c r="F116" s="2" t="n">
@@ -3570,7 +3550,11 @@
           <t>O80 Investigation and security activities</t>
         </is>
       </c>
-      <c r="E117" s="2" t="n"/>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>T95 Repair and maintenance of computers, personal and household goods, and motor vehicles and motorcycles</t>
+        </is>
+      </c>
       <c r="F117" s="2" t="n">
         <v>207</v>
       </c>
@@ -3594,7 +3578,11 @@
           <t>N72 Scientific research and development</t>
         </is>
       </c>
-      <c r="E118" s="2" t="n"/>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>O82 Office administrative, office support and other business support activities</t>
+        </is>
+      </c>
       <c r="F118" s="2" t="n">
         <v>134</v>
       </c>
@@ -3670,11 +3658,7 @@
           <t>R88 Social work activities without accommodation</t>
         </is>
       </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>R86 Human health activities</t>
-        </is>
-      </c>
+      <c r="E121" s="2" t="n"/>
       <c r="F121" s="2" t="n">
         <v>5</v>
       </c>
@@ -3695,14 +3679,10 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>T96 Personal service activities</t>
-        </is>
-      </c>
-      <c r="E122" s="2" t="inlineStr">
-        <is>
-          <t>O78 Employment activities</t>
-        </is>
-      </c>
+          <t>Q85 Education</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="n"/>
       <c r="F122" s="2" t="n">
         <v>16</v>
       </c>
@@ -3747,14 +3727,10 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>N74 Other professional, scientific and technical activities</t>
-        </is>
-      </c>
-      <c r="E124" s="2" t="inlineStr">
-        <is>
-          <t>N72 Scientific research and development</t>
-        </is>
-      </c>
+          <t>R86 Human health activities</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="n"/>
       <c r="F124" s="2" t="n">
         <v>10</v>
       </c>
@@ -3778,11 +3754,7 @@
           <t>I56 Food and beverage service activities</t>
         </is>
       </c>
-      <c r="E125" s="2" t="inlineStr">
-        <is>
-          <t>C10 Manufacture of food products</t>
-        </is>
-      </c>
+      <c r="E125" s="2" t="n"/>
       <c r="F125" s="2" t="n">
         <v>8</v>
       </c>
@@ -3855,7 +3827,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>L64 Financial service activities, except insurance and pension funding</t>
+          <t>L65 Insurance, reinsurance and pension funding, except compulsory social security</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -3883,12 +3855,12 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>K62 Computer programming, consultancy and related activities</t>
         </is>
       </c>
       <c r="F129" s="2" t="n">
@@ -3911,7 +3883,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>C19 Manufacture of coke and refined petroleum products</t>
+          <t>F43 Specialized construction activities</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -3939,12 +3911,12 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
+          <t>P84 Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
           <t>I56 Food and beverage service activities</t>
-        </is>
-      </c>
-      <c r="E131" s="2" t="inlineStr">
-        <is>
-          <t>O81 Services to buildings and landscape activities</t>
         </is>
       </c>
       <c r="F131" s="2" t="n">
@@ -3998,7 +3970,11 @@
           <t>R86 Human health activities</t>
         </is>
       </c>
-      <c r="E133" s="2" t="n"/>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>R87 Residential care activities</t>
+        </is>
+      </c>
       <c r="F133" s="2" t="n">
         <v>4</v>
       </c>
@@ -4052,7 +4028,7 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>N74 Other professional, scientific and technical activities</t>
+          <t>K62 Computer programming, consultancy and related activities</t>
         </is>
       </c>
       <c r="F135" s="2" t="n">
@@ -4102,11 +4078,7 @@
           <t>R87 Residential care activities</t>
         </is>
       </c>
-      <c r="E137" s="2" t="inlineStr">
-        <is>
-          <t>R86 Human health activities</t>
-        </is>
-      </c>
+      <c r="E137" s="2" t="n"/>
       <c r="F137" s="2" t="n">
         <v>13</v>
       </c>
@@ -4130,7 +4102,11 @@
           <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
-      <c r="E138" s="2" t="n"/>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>O81 Services to buildings and landscape activities</t>
+        </is>
+      </c>
       <c r="F138" s="2" t="n">
         <v>31</v>
       </c>
@@ -4151,12 +4127,12 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>A02 Forestry and logging</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>A03 Fishing and aquaculture</t>
+          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
         </is>
       </c>
       <c r="F139" s="2" t="n">
@@ -4179,12 +4155,12 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
+          <t>U97 Activities of households as employers of domestic personnel</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
           <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
-        </is>
-      </c>
-      <c r="E140" s="2" t="inlineStr">
-        <is>
-          <t>E39 Remediation and other waste management service activities</t>
         </is>
       </c>
       <c r="F140" s="2" t="n">
@@ -4210,7 +4186,11 @@
           <t>R86 Human health activities</t>
         </is>
       </c>
-      <c r="E141" s="2" t="n"/>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
+        </is>
+      </c>
       <c r="F141" s="2" t="n">
         <v>9</v>
       </c>
@@ -4231,12 +4211,12 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
+          <t>F42 Civil engineering</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
           <t>F43 Specialized construction activities</t>
-        </is>
-      </c>
-      <c r="E142" s="2" t="inlineStr">
-        <is>
-          <t>F41 Construction of residential and non-residential buildings</t>
         </is>
       </c>
       <c r="F142" s="2" t="n">
@@ -4259,12 +4239,12 @@
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>O82 Office administrative, office support and other business support activities</t>
+          <t>S91 Library, archives, museum and other cultural activities</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
+          <t>A01 Crop and animal production, hunting and related service activities</t>
         </is>
       </c>
       <c r="F143" s="2" t="n">
@@ -4290,7 +4270,11 @@
           <t>R86 Human health activities</t>
         </is>
       </c>
-      <c r="E144" s="2" t="n"/>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>P84 Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
       <c r="F144" s="2" t="n">
         <v>5</v>
       </c>
@@ -4335,12 +4319,12 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>C17 Manufacture of paper and paper products</t>
+          <t>T94 Activities of membership organizations</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>T94 Activities of membership organizations</t>
+          <t>P84 Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F146" s="2" t="n">
@@ -4363,14 +4347,10 @@
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>O81 Services to buildings and landscape activities</t>
-        </is>
-      </c>
-      <c r="E147" s="2" t="inlineStr">
-        <is>
           <t>F42 Civil engineering</t>
         </is>
       </c>
+      <c r="E147" s="2" t="n"/>
       <c r="F147" s="2" t="n">
         <v>53</v>
       </c>
@@ -4391,12 +4371,12 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>T96 Personal service activities</t>
+          <t>O82 Office administrative, office support and other business support activities</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>O78 Employment activities</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="F148" s="2" t="n">
@@ -4422,7 +4402,11 @@
           <t>S91 Library, archives, museum and other cultural activities</t>
         </is>
       </c>
-      <c r="E149" s="2" t="n"/>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>F42 Civil engineering</t>
+        </is>
+      </c>
       <c r="F149" s="2" t="n">
         <v>18</v>
       </c>
@@ -4495,12 +4479,12 @@
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
+          <t>P84 Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
           <t>O80 Investigation and security activities</t>
-        </is>
-      </c>
-      <c r="E152" s="2" t="inlineStr">
-        <is>
-          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
         </is>
       </c>
       <c r="F152" s="2" t="n">
@@ -4528,7 +4512,7 @@
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>J58 Publishing activities</t>
+          <t>N74 Other professional, scientific and technical activities</t>
         </is>
       </c>
       <c r="F153" s="2" t="n">
@@ -4554,7 +4538,11 @@
           <t>O82 Office administrative, office support and other business support activities</t>
         </is>
       </c>
-      <c r="E154" s="2" t="n"/>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>B09 Mining support service activities</t>
+        </is>
+      </c>
       <c r="F154" s="2" t="n">
         <v>31</v>
       </c>
@@ -4651,12 +4639,12 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
+          <t>G47 Retail trade</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
           <t>I56 Food and beverage service activities</t>
-        </is>
-      </c>
-      <c r="E158" s="2" t="inlineStr">
-        <is>
-          <t>G47 Retail trade</t>
         </is>
       </c>
       <c r="F158" s="2" t="n">
@@ -4684,7 +4672,7 @@
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>P84 Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F159" s="2" t="n">
@@ -4710,11 +4698,7 @@
           <t>N72 Scientific research and development</t>
         </is>
       </c>
-      <c r="E160" s="2" t="inlineStr">
-        <is>
-          <t>N73 Activities of advertising, market research and public relations</t>
-        </is>
-      </c>
+      <c r="E160" s="2" t="n"/>
       <c r="F160" s="2" t="n">
         <v>7</v>
       </c>
@@ -4735,12 +4719,12 @@
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>O81 Services to buildings and landscape activities</t>
+          <t>N74 Other professional, scientific and technical activities</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="F161" s="2" t="n">
@@ -4763,12 +4747,12 @@
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
+          <t>S90 Arts creation and performing arts activities</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
           <t>O82 Office administrative, office support and other business support activities</t>
-        </is>
-      </c>
-      <c r="E162" s="2" t="inlineStr">
-        <is>
-          <t>S90 Arts creation and performing arts activities</t>
         </is>
       </c>
       <c r="F162" s="2" t="n">
@@ -4815,12 +4799,12 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
+          <t>N73 Activities of advertising, market research and public relations</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
           <t>Q85 Education</t>
-        </is>
-      </c>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t>N73 Activities of advertising, market research and public relations</t>
         </is>
       </c>
       <c r="F164" s="2" t="n">
@@ -4843,12 +4827,12 @@
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
+          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
           <t>R88 Social work activities without accommodation</t>
-        </is>
-      </c>
-      <c r="E165" s="2" t="inlineStr">
-        <is>
-          <t>T96 Personal service activities</t>
         </is>
       </c>
       <c r="F165" s="2" t="n">
@@ -4874,11 +4858,7 @@
           <t>Q85 Education</t>
         </is>
       </c>
-      <c r="E166" s="2" t="inlineStr">
-        <is>
-          <t>M68 Real estate activities</t>
-        </is>
-      </c>
+      <c r="E166" s="2" t="n"/>
       <c r="F166" s="2" t="n">
         <v>189</v>
       </c>
@@ -4927,12 +4907,12 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
+          <t>P84 Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
           <t>Q85 Education</t>
-        </is>
-      </c>
-      <c r="E168" s="2" t="inlineStr">
-        <is>
-          <t>C15 Manufacture of leather and related products</t>
         </is>
       </c>
       <c r="F168" s="2" t="n">
@@ -4960,7 +4940,7 @@
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>R87 Residential care activities</t>
+          <t>P84 Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F169" s="2" t="n">
@@ -4988,7 +4968,7 @@
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>S91 Library, archives, museum and other cultural activities</t>
+          <t>L64 Financial service activities, except insurance and pension funding</t>
         </is>
       </c>
       <c r="F170" s="2" t="n">
@@ -5011,14 +4991,10 @@
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>J60 Programming, broadcasting, news agency and other content distribution activities</t>
-        </is>
-      </c>
-      <c r="E171" s="2" t="inlineStr">
-        <is>
-          <t>J58 Publishing activities</t>
-        </is>
-      </c>
+          <t>R88 Social work activities without accommodation</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="n"/>
       <c r="F171" s="2" t="n">
         <v>3</v>
       </c>
@@ -5039,14 +5015,10 @@
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>R87 Residential care activities</t>
-        </is>
-      </c>
-      <c r="E172" s="2" t="inlineStr">
-        <is>
           <t>R86 Human health activities</t>
         </is>
       </c>
+      <c r="E172" s="2" t="n"/>
       <c r="F172" s="2" t="n">
         <v>5</v>
       </c>
@@ -5067,7 +5039,7 @@
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>U98 Undifferentiated goods- and services-producing activities of private households for own use</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="E173" s="2" t="n"/>
@@ -5124,7 +5096,7 @@
       </c>
       <c r="E175" s="2" t="inlineStr">
         <is>
-          <t>K61 Telecommunications</t>
+          <t>R87 Residential care activities</t>
         </is>
       </c>
       <c r="F175" s="2" t="n">
@@ -5150,11 +5122,7 @@
           <t>R87 Residential care activities</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
-        <is>
-          <t>O82 Office administrative, office support and other business support activities</t>
-        </is>
-      </c>
+      <c r="E176" s="2" t="n"/>
       <c r="F176" s="2" t="n">
         <v>31</v>
       </c>
@@ -5175,12 +5143,12 @@
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>N72 Scientific research and development</t>
+          <t>R87 Residential care activities</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
         <is>
-          <t>R87 Residential care activities</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="F177" s="2" t="n">
@@ -5231,14 +5199,10 @@
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>R87 Residential care activities</t>
-        </is>
-      </c>
-      <c r="E179" s="2" t="inlineStr">
-        <is>
-          <t>R86 Human health activities</t>
-        </is>
-      </c>
+          <t>Q85 Education</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="n"/>
       <c r="F179" s="2" t="n">
         <v>25</v>
       </c>
@@ -5290,7 +5254,11 @@
           <t>T95 Repair and maintenance of computers, personal and household goods, and motor vehicles and motorcycles</t>
         </is>
       </c>
-      <c r="E181" s="2" t="n"/>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
+        </is>
+      </c>
       <c r="F181" s="2" t="n">
         <v>41</v>
       </c>
@@ -5311,7 +5279,7 @@
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>O82 Office administrative, office support and other business support activities</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="E182" s="2" t="n"/>
@@ -5338,7 +5306,11 @@
           <t>O81 Services to buildings and landscape activities</t>
         </is>
       </c>
-      <c r="E183" s="2" t="n"/>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>P84 Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
       <c r="F183" s="2" t="n">
         <v>19</v>
       </c>
@@ -5359,14 +5331,10 @@
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>E36 Water collection, treatment and supply</t>
-        </is>
-      </c>
-      <c r="E184" s="2" t="inlineStr">
-        <is>
-          <t>E39 Remediation and other waste management service activities</t>
-        </is>
-      </c>
+          <t>O78 Employment activities</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="n"/>
       <c r="F184" s="2" t="n">
         <v>77</v>
       </c>
@@ -5390,7 +5358,11 @@
           <t>R86 Human health activities</t>
         </is>
       </c>
-      <c r="E185" s="2" t="n"/>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>O78 Employment activities</t>
+        </is>
+      </c>
       <c r="F185" s="2" t="n">
         <v>59</v>
       </c>
@@ -5416,7 +5388,7 @@
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>H50 Water transport</t>
         </is>
       </c>
       <c r="F186" s="2" t="n">
@@ -5442,7 +5414,11 @@
           <t>R86 Human health activities</t>
         </is>
       </c>
-      <c r="E187" s="2" t="n"/>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>Q85 Education</t>
+        </is>
+      </c>
       <c r="F187" s="2" t="n">
         <v>5</v>
       </c>
@@ -5494,11 +5470,7 @@
           <t>R87 Residential care activities</t>
         </is>
       </c>
-      <c r="E189" s="2" t="inlineStr">
-        <is>
-          <t>R86 Human health activities</t>
-        </is>
-      </c>
+      <c r="E189" s="2" t="n"/>
       <c r="F189" s="2" t="n">
         <v>36</v>
       </c>
@@ -5522,11 +5494,7 @@
           <t>E36 Water collection, treatment and supply</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
-        <is>
-          <t>E37 Sewerage</t>
-        </is>
-      </c>
+      <c r="E190" s="2" t="n"/>
       <c r="F190" s="2" t="n">
         <v>8</v>
       </c>
@@ -5550,11 +5518,7 @@
           <t>S93 Sports activities and amusement and recreation activities</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
-        <is>
-          <t>S92 Gambling and betting activities</t>
-        </is>
-      </c>
+      <c r="E191" s="2" t="n"/>
       <c r="F191" s="2" t="n">
         <v>52</v>
       </c>
@@ -5658,7 +5622,11 @@
           <t>Q85 Education</t>
         </is>
       </c>
-      <c r="E195" s="2" t="n"/>
+      <c r="E195" s="2" t="inlineStr">
+        <is>
+          <t>J59 Motion picture, video and television programme production, sound recording and music publishing activities</t>
+        </is>
+      </c>
       <c r="F195" s="2" t="n">
         <v>8</v>
       </c>
@@ -5707,12 +5675,12 @@
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
+          <t>R86 Human health activities</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="inlineStr">
+        <is>
           <t>R88 Social work activities without accommodation</t>
-        </is>
-      </c>
-      <c r="E197" s="2" t="inlineStr">
-        <is>
-          <t>S91 Library, archives, museum and other cultural activities</t>
         </is>
       </c>
       <c r="F197" s="2" t="n">
@@ -5759,12 +5727,12 @@
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>R88 Social work activities without accommodation</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>P84 Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F199" s="2" t="n">
@@ -5790,7 +5758,11 @@
           <t>S91 Library, archives, museum and other cultural activities</t>
         </is>
       </c>
-      <c r="E200" s="2" t="n"/>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>M68 Real estate activities</t>
+        </is>
+      </c>
       <c r="F200" s="2" t="n">
         <v>34</v>
       </c>
@@ -5811,7 +5783,7 @@
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>J60 Programming, broadcasting, news agency and other content distribution activities</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="E201" s="2" t="inlineStr">
@@ -5839,12 +5811,12 @@
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>U97 Activities of households as employers of domestic personnel</t>
+          <t>R88 Social work activities without accommodation</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>R88 Social work activities without accommodation</t>
+          <t>P84 Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F202" s="2" t="n">
@@ -5867,12 +5839,12 @@
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>C10 Manufacture of food products</t>
+          <t>N73 Activities of advertising, market research and public relations</t>
         </is>
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>C19 Manufacture of coke and refined petroleum products</t>
         </is>
       </c>
       <c r="F203" s="2" t="n">
@@ -5900,7 +5872,7 @@
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
+          <t>J58 Publishing activities</t>
         </is>
       </c>
       <c r="F204" s="2" t="n">
@@ -5923,12 +5895,12 @@
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
+          <t>T95 Repair and maintenance of computers, personal and household goods, and motor vehicles and motorcycles</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
           <t>C33 Repair, maintenance and installation of machinery and equipment</t>
-        </is>
-      </c>
-      <c r="E205" s="2" t="inlineStr">
-        <is>
-          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="F205" s="2" t="n">
@@ -5954,11 +5926,7 @@
           <t>L64 Financial service activities, except insurance and pension funding</t>
         </is>
       </c>
-      <c r="E206" s="2" t="inlineStr">
-        <is>
-          <t>L66 Activities auxiliary to financial service and insurance activities</t>
-        </is>
-      </c>
+      <c r="E206" s="2" t="n"/>
       <c r="F206" s="2" t="n">
         <v>4</v>
       </c>
@@ -6051,7 +6019,7 @@
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>Q85 Education</t>
         </is>
       </c>
       <c r="E210" s="2" t="n"/>
@@ -6095,12 +6063,12 @@
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
+          <t>O82 Office administrative, office support and other business support activities</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
           <t>J60 Programming, broadcasting, news agency and other content distribution activities</t>
-        </is>
-      </c>
-      <c r="E212" s="2" t="inlineStr">
-        <is>
-          <t>C15 Manufacture of leather and related products</t>
         </is>
       </c>
       <c r="F212" s="2" t="n">
@@ -6143,12 +6111,12 @@
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
+          <t>H49 Land transport and transport via pipelines</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
           <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
-        </is>
-      </c>
-      <c r="E214" s="2" t="inlineStr">
-        <is>
-          <t>H49 Land transport and transport via pipelines</t>
         </is>
       </c>
       <c r="F214" s="2" t="n">
@@ -6174,11 +6142,7 @@
           <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
-      <c r="E215" s="2" t="inlineStr">
-        <is>
-          <t>N73 Activities of advertising, market research and public relations</t>
-        </is>
-      </c>
+      <c r="E215" s="2" t="n"/>
       <c r="F215" s="2" t="n">
         <v>21</v>
       </c>
@@ -6199,12 +6163,12 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
+          <t>T95 Repair and maintenance of computers, personal and household goods, and motor vehicles and motorcycles</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
           <t>C33 Repair, maintenance and installation of machinery and equipment</t>
-        </is>
-      </c>
-      <c r="E216" s="2" t="inlineStr">
-        <is>
-          <t>T95 Repair and maintenance of computers, personal and household goods, and motor vehicles and motorcycles</t>
         </is>
       </c>
       <c r="F216" s="2" t="n">
@@ -6230,11 +6194,7 @@
           <t>K62 Computer programming, consultancy and related activities</t>
         </is>
       </c>
-      <c r="E217" s="2" t="inlineStr">
-        <is>
-          <t>C15 Manufacture of leather and related products</t>
-        </is>
-      </c>
+      <c r="E217" s="2" t="n"/>
       <c r="F217" s="2" t="n">
         <v>24</v>
       </c>
@@ -6255,7 +6215,7 @@
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>O82 Office administrative, office support and other business support activities</t>
+          <t>C10 Manufacture of food products</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
@@ -6286,7 +6246,11 @@
           <t>O82 Office administrative, office support and other business support activities</t>
         </is>
       </c>
-      <c r="E219" s="2" t="n"/>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>B09 Mining support service activities</t>
+        </is>
+      </c>
       <c r="F219" s="2" t="n">
         <v>4</v>
       </c>
@@ -6310,7 +6274,11 @@
           <t>T94 Activities of membership organizations</t>
         </is>
       </c>
-      <c r="E220" s="2" t="n"/>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>O82 Office administrative, office support and other business support activities</t>
+        </is>
+      </c>
       <c r="F220" s="2" t="n">
         <v>3</v>
       </c>
@@ -6331,7 +6299,7 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>R88 Social work activities without accommodation</t>
+          <t>R86 Human health activities</t>
         </is>
       </c>
       <c r="E221" s="2" t="inlineStr">
@@ -6392,7 +6360,7 @@
       </c>
       <c r="E223" s="2" t="inlineStr">
         <is>
-          <t>F42 Civil engineering</t>
+          <t>N72 Scientific research and development</t>
         </is>
       </c>
       <c r="F223" s="2" t="n">
@@ -6439,12 +6407,12 @@
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>N72 Scientific research and development</t>
+          <t>B06 Extraction of crude petroleum and natural gas</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
         <is>
-          <t>B06 Extraction of crude petroleum and natural gas</t>
+          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F225" s="2" t="n">
@@ -6494,7 +6462,11 @@
           <t>R86 Human health activities</t>
         </is>
       </c>
-      <c r="E227" s="2" t="n"/>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
+        </is>
+      </c>
       <c r="F227" s="2" t="n">
         <v>7</v>
       </c>
@@ -6518,11 +6490,7 @@
           <t>I56 Food and beverage service activities</t>
         </is>
       </c>
-      <c r="E228" s="2" t="inlineStr">
-        <is>
-          <t>C10 Manufacture of food products</t>
-        </is>
-      </c>
+      <c r="E228" s="2" t="n"/>
       <c r="F228" s="2" t="n">
         <v>29</v>
       </c>
@@ -6543,14 +6511,10 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>R86 Human health activities</t>
-        </is>
-      </c>
-      <c r="E229" s="2" t="inlineStr">
-        <is>
-          <t>N73 Activities of advertising, market research and public relations</t>
-        </is>
-      </c>
+          <t>N72 Scientific research and development</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="n"/>
       <c r="F229" s="2" t="n">
         <v>28</v>
       </c>
@@ -6571,12 +6535,12 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
+          <t>E36 Water collection, treatment and supply</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
           <t>R86 Human health activities</t>
-        </is>
-      </c>
-      <c r="E230" s="2" t="inlineStr">
-        <is>
-          <t>R87 Residential care activities</t>
         </is>
       </c>
       <c r="F230" s="2" t="n">
@@ -6604,7 +6568,7 @@
       </c>
       <c r="E231" s="2" t="inlineStr">
         <is>
-          <t>S91 Library, archives, museum and other cultural activities</t>
+          <t>C30 Manufacture of other transport equipment</t>
         </is>
       </c>
       <c r="F231" s="2" t="n">
@@ -6632,7 +6596,7 @@
       </c>
       <c r="E232" s="2" t="inlineStr">
         <is>
-          <t>J60 Programming, broadcasting, news agency and other content distribution activities</t>
+          <t>K63 Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F232" s="2" t="n">
@@ -6658,7 +6622,11 @@
           <t>O82 Office administrative, office support and other business support activities</t>
         </is>
       </c>
-      <c r="E233" s="2" t="n"/>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>B09 Mining support service activities</t>
+        </is>
+      </c>
       <c r="F233" s="2" t="n">
         <v>15</v>
       </c>

</xml_diff>